<commit_message>
Add language. Remove series.
</commit_message>
<xml_diff>
--- a/tests/fixtures/invalid_books.xlsx
+++ b/tests/fixtures/invalid_books.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,50 +444,45 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Series</t>
+          <t>Language</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Series Number</t>
+          <t>Publisher</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Publisher</t>
+          <t>Publication Year</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Publication Year</t>
+          <t>Shelf</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Shelf</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Tags</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Tags</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Rating</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
-        <is>
-          <t>Rating</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
         <is>
           <t>Cover Image</t>
         </is>
@@ -509,10 +504,8 @@
           <t>Frank Herbert</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>9780441013593</t>
-        </is>
+      <c r="D2" t="n">
+        <v>9780441013593</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -520,33 +513,32 @@
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Ace Books</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="H2" t="n">
         <v>1965</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
           <t>favorites</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -564,10 +556,8 @@
           <t>Frank Herbert</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>9780441013593</t>
-        </is>
+      <c r="D3" t="n">
+        <v>9780441013593</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -575,29 +565,28 @@
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Ace Books</t>
         </is>
       </c>
-      <c r="I3" t="n">
+      <c r="H3" t="n">
         <v>1965</v>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
           <t>Available</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -619,20 +608,19 @@
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="n">
+      <c r="H4" t="n">
         <v>1951</v>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -658,20 +646,19 @@
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="n">
+      <c r="H5" t="n">
         <v>1937</v>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Checked Out</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -689,10 +676,8 @@
           <t>Isaac Asimov</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>9780553293357</t>
-        </is>
+      <c r="D6" t="n">
+        <v>9780553293357</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -701,20 +686,19 @@
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="n">
+      <c r="H6" t="n">
         <v>1951</v>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -732,10 +716,8 @@
           <t>William Gibson</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>9780553293357</t>
-        </is>
+      <c r="D7" t="n">
+        <v>9780553293357</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -744,20 +726,19 @@
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="n">
+      <c r="H7" t="n">
         <v>1984</v>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>